<commit_message>
Correct the mirror finding: overnight lag, not a broken sync
I labelled the three Dagelijkse Groenmarkt rows BOT OUT OF SYNC. Checking
the middle of the pipeline showed that was too strong.

bot.ticket_taxonomy already held Freshdesk's current numbers
(EUR74/67/60/89, synced 02:00), so Freshdesk -> taxonomy is working. Only
bot.form_schemas still had EUR69/62/55, from the 04:00 refresh the previous
day. The pipeline is two nightly stages and the mirror was one cycle behind,
not broken.

It still matters and still belongs in the sheet: an edit made just after
02:00 is quoted stale for up to about 26 hours, and the outbound price
guard validates against the mirror, so during that window it protects the
stale number rather than the form. The row now says so, and says what to do
if it survives two nights.
</commit_message>
<xml_diff>
--- a/docs/club-pricing-comparison.xlsx
+++ b/docs/club-pricing-comparison.xlsx
@@ -520,7 +520,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>bot.form_schemas in Supabase. The bot does NOT read Freshdesk — its "Fetch Form Options" node reads this mirror. Where this column disagrees with the form, the member is being told the wrong price and nobody has to decide anything: it is a sync bug. Those rows sort to the top of Differences.</t>
+          <t>bot.form_schemas in Supabase. The bot does NOT read Freshdesk — its "Fetch Form Options" node reads this mirror, fed nightly: Freshdesk → 02:00 ticket_taxonomy → 04:00 form_schemas. Where this column disagrees with the form it is usually LAG, not an error: an edit made just after 02:00 is quoted stale for up to about 26 hours. It still matters — for that window members hear a price the form no longer offers, and the bot's own price guard validates against this mirror, so it protects the stale number. If a row is still here after two nights it is not lag: check Bot - Refresh Form Options.</t>
         </is>
       </c>
     </row>
@@ -721,12 +721,12 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>BOT OUT OF SYNC</t>
+          <t>bot behind the form</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Bot quotes €69, the form says €74 — resync bot.form_schemas</t>
+          <t>Bot quotes €69, the form says €74. Usually overnight lag — if it is still here after two nights, check Bot - Refresh Form Options</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -768,12 +768,12 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>BOT OUT OF SYNC</t>
+          <t>bot behind the form</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Bot quotes €62, the form says €67 — resync bot.form_schemas</t>
+          <t>Bot quotes €62, the form says €67. Usually overnight lag — if it is still here after two nights, check Bot - Refresh Form Options</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -815,12 +815,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>BOT OUT OF SYNC</t>
+          <t>bot behind the form</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Bot quotes €55, the form says €60 — resync bot.form_schemas</t>
+          <t>Bot quotes €55, the form says €60. Usually overnight lag — if it is still here after two nights, check Bot - Refresh Form Options</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
@@ -20220,12 +20220,12 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>BOT OUT OF SYNC</t>
+          <t>bot behind the form</t>
         </is>
       </c>
       <c r="H270" s="6" t="inlineStr">
         <is>
-          <t>Bot quotes €69, the form says €74 — resync bot.form_schemas</t>
+          <t>Bot quotes €69, the form says €74. Usually overnight lag — if it is still here after two nights, check Bot - Refresh Form Options</t>
         </is>
       </c>
       <c r="I270" s="7" t="inlineStr">
@@ -20267,12 +20267,12 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>BOT OUT OF SYNC</t>
+          <t>bot behind the form</t>
         </is>
       </c>
       <c r="H271" s="6" t="inlineStr">
         <is>
-          <t>Bot quotes €62, the form says €67 — resync bot.form_schemas</t>
+          <t>Bot quotes €62, the form says €67. Usually overnight lag — if it is still here after two nights, check Bot - Refresh Form Options</t>
         </is>
       </c>
       <c r="I271" s="7" t="inlineStr">
@@ -20314,12 +20314,12 @@
       </c>
       <c r="G272" s="5" t="inlineStr">
         <is>
-          <t>BOT OUT OF SYNC</t>
+          <t>bot behind the form</t>
         </is>
       </c>
       <c r="H272" s="6" t="inlineStr">
         <is>
-          <t>Bot quotes €55, the form says €60 — resync bot.form_schemas</t>
+          <t>Bot quotes €55, the form says €60. Usually overnight lag — if it is still here after two nights, check Bot - Refresh Form Options</t>
         </is>
       </c>
       <c r="I272" s="7" t="inlineStr">

</xml_diff>